<commit_message>
Fixed bug 2 and 3
</commit_message>
<xml_diff>
--- a/output/teacher_timetables_even.xlsx
+++ b/output/teacher_timetables_even.xlsx
@@ -96,10 +96,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -617,34 +617,10 @@
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr"/>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>CS501 LEC
-(CSE_4_B)
-Room: 101</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>CS501 LEC
-(CSE_4_B)
-Room: 101</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>CS501 LEC
-(CSE_4_B)
-Room: 101</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>CS501 LEC
-(CSE_4_B)
-Room: 101</t>
-        </is>
-      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="3" t="inlineStr"/>
       <c r="I3" s="3" t="inlineStr"/>
@@ -662,31 +638,31 @@
       <c r="U3" s="3" t="inlineStr"/>
     </row>
     <row r="4" ht="35" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr"/>
-      <c r="I4" s="5" t="inlineStr"/>
-      <c r="J4" s="5" t="inlineStr"/>
-      <c r="K4" s="5" t="inlineStr"/>
-      <c r="L4" s="5" t="inlineStr"/>
-      <c r="M4" s="5" t="inlineStr"/>
-      <c r="N4" s="5" t="inlineStr"/>
-      <c r="O4" s="5" t="inlineStr"/>
-      <c r="P4" s="5" t="inlineStr"/>
-      <c r="Q4" s="5" t="inlineStr"/>
-      <c r="R4" s="5" t="inlineStr"/>
-      <c r="S4" s="5" t="inlineStr"/>
-      <c r="T4" s="5" t="inlineStr"/>
-      <c r="U4" s="5" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr"/>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr"/>
+      <c r="N4" s="4" t="inlineStr"/>
+      <c r="O4" s="4" t="inlineStr"/>
+      <c r="P4" s="4" t="inlineStr"/>
+      <c r="Q4" s="4" t="inlineStr"/>
+      <c r="R4" s="4" t="inlineStr"/>
+      <c r="S4" s="4" t="inlineStr"/>
+      <c r="T4" s="4" t="inlineStr"/>
+      <c r="U4" s="4" t="inlineStr"/>
     </row>
     <row r="5" ht="35" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -716,31 +692,55 @@
       <c r="U5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="35" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr"/>
-      <c r="J6" s="5" t="inlineStr"/>
-      <c r="K6" s="5" t="inlineStr"/>
-      <c r="L6" s="5" t="inlineStr"/>
-      <c r="M6" s="5" t="inlineStr"/>
-      <c r="N6" s="5" t="inlineStr"/>
-      <c r="O6" s="5" t="inlineStr"/>
-      <c r="P6" s="5" t="inlineStr"/>
-      <c r="Q6" s="5" t="inlineStr"/>
-      <c r="R6" s="5" t="inlineStr"/>
-      <c r="S6" s="5" t="inlineStr"/>
-      <c r="T6" s="5" t="inlineStr"/>
-      <c r="U6" s="5" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>CS501 LEC
+(CSE_4_B)
+Room: 101</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>CS501 LEC
+(CSE_4_B)
+Room: 101</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>CS501 LEC
+(CSE_4_B)
+Room: 101</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>CS501 LEC
+(CSE_4_B)
+Room: 101</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr"/>
+      <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr"/>
+      <c r="L6" s="4" t="inlineStr"/>
+      <c r="M6" s="4" t="inlineStr"/>
+      <c r="N6" s="4" t="inlineStr"/>
+      <c r="O6" s="4" t="inlineStr"/>
+      <c r="P6" s="4" t="inlineStr"/>
+      <c r="Q6" s="4" t="inlineStr"/>
+      <c r="R6" s="4" t="inlineStr"/>
+      <c r="S6" s="4" t="inlineStr"/>
+      <c r="T6" s="4" t="inlineStr"/>
+      <c r="U6" s="4" t="inlineStr"/>
     </row>
     <row r="7" ht="35" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -941,77 +941,83 @@
       <c r="K3" s="3" t="inlineStr"/>
       <c r="L3" s="3" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
-      <c r="N3" s="3" t="inlineStr"/>
-      <c r="O3" s="3" t="inlineStr"/>
-      <c r="P3" s="3" t="inlineStr"/>
-      <c r="Q3" s="4" t="inlineStr">
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>CS502 LEC
 (CSE_4_B)
-Room: 101</t>
-        </is>
-      </c>
-      <c r="R3" s="4" t="inlineStr">
+Room: 102</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>CS502 LEC
 (CSE_4_B)
-Room: 101</t>
-        </is>
-      </c>
-      <c r="S3" s="4" t="inlineStr">
+Room: 102</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>CS502 LEC
 (CSE_4_B)
-Room: 101</t>
-        </is>
-      </c>
+Room: 102</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr"/>
+      <c r="R3" s="3" t="inlineStr"/>
+      <c r="S3" s="3" t="inlineStr"/>
       <c r="T3" s="3" t="inlineStr"/>
       <c r="U3" s="3" t="inlineStr"/>
     </row>
     <row r="4" ht="35" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr"/>
-      <c r="I4" s="5" t="inlineStr"/>
-      <c r="J4" s="5" t="inlineStr"/>
-      <c r="K4" s="5" t="inlineStr"/>
-      <c r="L4" s="5" t="inlineStr"/>
-      <c r="M4" s="5" t="inlineStr"/>
-      <c r="N4" s="5" t="inlineStr"/>
-      <c r="O4" s="5" t="inlineStr"/>
-      <c r="P4" s="5" t="inlineStr"/>
-      <c r="Q4" s="4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr"/>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>CS502 LEC
 (CSE_4_B)
-Room: 101</t>
-        </is>
-      </c>
-      <c r="R4" s="4" t="inlineStr">
+Room: 102</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>CS502 LEC
 (CSE_4_B)
-Room: 101</t>
-        </is>
-      </c>
-      <c r="S4" s="4" t="inlineStr">
+Room: 102</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>CS502 LEC
 (CSE_4_B)
-Room: 101</t>
-        </is>
-      </c>
-      <c r="T4" s="5" t="inlineStr"/>
-      <c r="U4" s="5" t="inlineStr"/>
+Room: 102</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>CS502 LEC
+(CSE_4_B)
+Room: 102</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr"/>
+      <c r="N4" s="4" t="inlineStr"/>
+      <c r="O4" s="4" t="inlineStr"/>
+      <c r="P4" s="4" t="inlineStr"/>
+      <c r="Q4" s="4" t="inlineStr"/>
+      <c r="R4" s="4" t="inlineStr"/>
+      <c r="S4" s="4" t="inlineStr"/>
+      <c r="T4" s="4" t="inlineStr"/>
+      <c r="U4" s="4" t="inlineStr"/>
     </row>
     <row r="5" ht="35" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -1020,7 +1026,13 @@
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr"/>
-      <c r="C5" s="3" t="inlineStr"/>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>CS502 TUT
+(CSE_4_B)
+Room: 102</t>
+        </is>
+      </c>
       <c r="D5" s="3" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr"/>
@@ -1041,31 +1053,31 @@
       <c r="U5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="35" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr"/>
-      <c r="J6" s="5" t="inlineStr"/>
-      <c r="K6" s="5" t="inlineStr"/>
-      <c r="L6" s="5" t="inlineStr"/>
-      <c r="M6" s="5" t="inlineStr"/>
-      <c r="N6" s="5" t="inlineStr"/>
-      <c r="O6" s="5" t="inlineStr"/>
-      <c r="P6" s="5" t="inlineStr"/>
-      <c r="Q6" s="5" t="inlineStr"/>
-      <c r="R6" s="5" t="inlineStr"/>
-      <c r="S6" s="5" t="inlineStr"/>
-      <c r="T6" s="5" t="inlineStr"/>
-      <c r="U6" s="5" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr"/>
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr"/>
+      <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr"/>
+      <c r="L6" s="4" t="inlineStr"/>
+      <c r="M6" s="4" t="inlineStr"/>
+      <c r="N6" s="4" t="inlineStr"/>
+      <c r="O6" s="4" t="inlineStr"/>
+      <c r="P6" s="4" t="inlineStr"/>
+      <c r="Q6" s="4" t="inlineStr"/>
+      <c r="R6" s="4" t="inlineStr"/>
+      <c r="S6" s="4" t="inlineStr"/>
+      <c r="T6" s="4" t="inlineStr"/>
+      <c r="U6" s="4" t="inlineStr"/>
     </row>
     <row r="7" ht="35" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -1075,27 +1087,9 @@
       </c>
       <c r="B7" s="3" t="inlineStr"/>
       <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>CS502 TUT
-(CSE_4_B)
-Room: 102</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>CS502 TUT
-(CSE_4_B)
-Room: 102</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>CS502 TUT
-(CSE_4_B)
-Room: 102</t>
-        </is>
-      </c>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr"/>

</xml_diff>